<commit_message>
🤖 [Archivio Semplificato] Spostati 1 titoli
</commit_message>
<xml_diff>
--- a/Storico_assegni.xlsx
+++ b/Storico_assegni.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,6 +548,46 @@
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>Versato OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>RICCARDO ROSSO</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>EA590017319S - TABACCHERIA RICEVITORIA VISENTINI PAOLO</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>0967584051</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>1717</v>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
         <is>
           <t>Versato OK</t>
         </is>

</xml_diff>